<commit_message>
Update Calendario Data Engineer V1.xlsx
</commit_message>
<xml_diff>
--- a/Calendario Data Engineer V1.xlsx
+++ b/Calendario Data Engineer V1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\diplomado-data-engineer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA958361-1B64-436F-A948-74EDFFCF4B2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B51273-CDF0-4CF3-8DD2-781565598FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5F69A3EF-6077-4BDE-A151-51A314216C0C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="77">
   <si>
     <t>Programa Diplomado
 Data Engineer versión 1 - 2026</t>
@@ -2193,6 +2193,9 @@
       <c r="D60" s="3">
         <v>3</v>
       </c>
+      <c r="E60" s="20" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A61" s="4">
@@ -2264,11 +2267,11 @@
       </c>
       <c r="E66">
         <f>SUMIF(E4:E63,"ok",D4:D63)</f>
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F66" s="27">
         <f>+E66/D66</f>
-        <v>0.92</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">

</xml_diff>